<commit_message>
Align roadmap phase one acceptance
</commit_message>
<xml_diff>
--- a/documentation/ryu-roadmap-example/ryu-internal-product-roadmap-example.xlsx
+++ b/documentation/ryu-roadmap-example/ryu-internal-product-roadmap-example.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R1fb822cbb1cf45b3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roadmap" sheetId="2" r:id="Rf55aa9c771fd4e00"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Plan" sheetId="3" r:id="R3bc6e2a7323f4f4a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Acceptance Matrix" sheetId="4" r:id="R92bb55e698794ca1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks &amp; Decisions" sheetId="5" r:id="R36112f6dc47a490d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Definitions" sheetId="6" r:id="Rb8ffbda301734706"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rd28747cd04d14b65"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roadmap" sheetId="2" r:id="R626cfca1634344f1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Plan" sheetId="3" r:id="Rca76a56645994ada"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Acceptance Matrix" sheetId="4" r:id="R4f59ae9d68424aab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks &amp; Decisions" sheetId="5" r:id="Rda22ecf40b0a49fa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Definitions" sheetId="6" r:id="Rc0c0c961a1c7427a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -529,7 +529,7 @@
       </x:c>
       <x:c r="B6" s="33" t="n">
         <x:f>COUNTIF(Roadmap!F2:F200,"Ready")+COUNTIF(Roadmap!F2:F200,"In Progress")</x:f>
-        <x:v>5</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -555,7 +555,7 @@
         <x:v>Next release</x:v>
       </x:c>
       <x:c r="B9" s="21" t="str">
-        <x:v>Release 1</x:v>
+        <x:v>Release 2</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -571,7 +571,7 @@
         <x:v>Last refreshed</x:v>
       </x:c>
       <x:c r="B11" s="34" t="n">
-        <x:v>46254</x:v>
+        <x:v>46280</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -604,11 +604,11 @@
       </x:c>
       <x:c r="C14" s="29" t="n">
         <x:f>COUNTIFS(Roadmap!B$2:B$200,A14,Roadmap!F$2:F$200,"Not Started")</x:f>
-        <x:v>2</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D14" s="29" t="n">
         <x:f>COUNTIFS(Roadmap!B$2:B$200,A14,Roadmap!F$2:F$200,"Ready")</x:f>
-        <x:v>2</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="E14" s="29" t="n">
         <x:f>COUNTIFS(Roadmap!B$2:B$200,A14,Roadmap!F$2:F$200,"In Progress")</x:f>
@@ -616,7 +616,7 @@
       </x:c>
       <x:c r="F14" s="19" t="n">
         <x:f>COUNTIFS(Roadmap!B$2:B$200,A14,Roadmap!F$2:F$200,"Done")</x:f>
-        <x:v>0</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -745,7 +745,7 @@
         <x:v>Notes</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" ht="56" customHeight="1">
+    <x:row r="2" ht="84" customHeight="1">
       <x:c r="A2" s="18" t="str">
         <x:v>R1-F01</x:v>
       </x:c>
@@ -762,7 +762,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="F2" s="29" t="str">
-        <x:v>Ready</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="G2" s="29" t="str">
         <x:v>Product</x:v>
@@ -780,19 +780,19 @@
         <x:v>Existing Ryu DB</x:v>
       </x:c>
       <x:c r="L2" s="29" t="str">
-        <x:v>Inventory current nodes, classify target systems, assign review depth, and agree on what must be rich versus thin.</x:v>
+        <x:v>Use the approved priority research queue to inventory existing systems, identify missing main systems and supporting relationship endpoints, assign rich versus thin or stub depth, and record the research order and owner.</x:v>
       </x:c>
       <x:c r="M2" s="29" t="str">
-        <x:v>Priority list is approved, each selected record has an owner and target review state, and deferred records are explicitly marked.</x:v>
+        <x:v>The approved queue names and orders the priority systems, assigns a primary worker, sets the target depth and review state, keeps supporting identities thin or stub, and records removals or deferrals.</x:v>
       </x:c>
       <x:c r="N2" s="29" t="str">
         <x:v>Spec Approved</x:v>
       </x:c>
       <x:c r="O2" s="19" t="str">
-        <x:v>Use this as the intake gate for content work.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3" ht="56" customHeight="1">
+        <x:v>The approved research queue and current production scope are documented.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="84" customHeight="1">
       <x:c r="A3" s="20" t="str">
         <x:v>R1-F02</x:v>
       </x:c>
@@ -803,13 +803,13 @@
         <x:v>Rich record backfill</x:v>
       </x:c>
       <x:c r="D3" s="30" t="str">
-        <x:v>Move selected priority systems from thin to rich records.</x:v>
+        <x:v>Apply the approved priority system batch as validated rich records.</x:v>
       </x:c>
       <x:c r="E3" s="30" t="str">
         <x:v>P0</x:v>
       </x:c>
       <x:c r="F3" s="30" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="G3" s="30" t="str">
         <x:v>Research</x:v>
@@ -827,19 +827,19 @@
         <x:v>R1-F01</x:v>
       </x:c>
       <x:c r="L3" s="30" t="str">
-        <x:v>Add summaries, operators, descriptions, source-backed access paths, identifiers, caveats, usage metrics, and review metadata.</x:v>
+        <x:v>Apply complete six-locale rich system aggregates through the Record API, including sourced profiles, approved descriptors, access guidance, metrics or explicit gaps, gallery evidence, and researched incident relationships. Preserve existing content, routes, sources, and review history.</x:v>
       </x:c>
       <x:c r="M3" s="30" t="str">
-        <x:v>At least six priority systems have source-backed rich records and no unresolved source refs in visible user-facing fields.</x:v>
+        <x:v>Every approved main record passes live validateOnly with a fresh precondition, applies and reads back exactly, has six complete agent_researched localizations, complete source-reference coverage, qualifying gallery evidence, and fully evidenced incident relationships; supporting identities remain thin or stub.</x:v>
       </x:c>
       <x:c r="N3" s="30" t="str">
         <x:v>QA Passed</x:v>
       </x:c>
       <x:c r="O3" s="21" t="str">
-        <x:v>Good first release demo because it makes Ryu visibly more useful.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4" ht="56" customHeight="1">
+        <x:v>Production application and readback completed 2026-09-11; OceanTeacher was later removed from system scope.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="84" customHeight="1">
       <x:c r="A4" s="20" t="str">
         <x:v>R1-F03</x:v>
       </x:c>
@@ -850,13 +850,13 @@
         <x:v>Data record visibility</x:v>
       </x:c>
       <x:c r="D4" s="30" t="str">
-        <x:v>Make data descriptors auditable from the UI.</x:v>
+        <x:v>Make approved data descriptors and their evidence auditable from User View.</x:v>
       </x:c>
       <x:c r="E4" s="30" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="F4" s="30" t="str">
-        <x:v>Ready</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="G4" s="30" t="str">
         <x:v>Frontend</x:v>
@@ -871,22 +871,22 @@
         <x:v>M</x:v>
       </x:c>
       <x:c r="K4" s="30" t="str">
-        <x:v>Data descriptors already exist</x:v>
+        <x:v>Approved system descriptor contract</x:v>
       </x:c>
       <x:c r="L4" s="30" t="str">
-        <x:v>Show descriptor IDs, descriptions, categories, and resolved source records from the existing details_json data descriptors.</x:v>
+        <x:v>Group descriptors by type, format, and standard in User View; show shared-vocabulary labels and localized descriptions with the resolved owner-local source title, URL, and accessed date. Show the localized standards research gap when none is assigned.</x:v>
       </x:c>
       <x:c r="M4" s="30" t="str">
-        <x:v>Reviewer can verify every visible data type, format, and standard without opening raw fields.</x:v>
+        <x:v>A reviewer can inspect each displayed descriptor's approved label, category, localized description, and resolved source evidence, or the standards gap, without opening Raw Fields.</x:v>
       </x:c>
       <x:c r="N4" s="30" t="str">
         <x:v>QA Passed</x:v>
       </x:c>
       <x:c r="O4" s="21" t="str">
-        <x:v>Mirrors the current cleanup tracker.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5" ht="56" customHeight="1">
+        <x:v>Production smoke verified FishBase standards and related record details.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="84" customHeight="1">
       <x:c r="A5" s="20" t="str">
         <x:v>R1-F04</x:v>
       </x:c>
@@ -897,13 +897,13 @@
         <x:v>Review trail surface</x:v>
       </x:c>
       <x:c r="D5" s="30" t="str">
-        <x:v>Expose record depth, review history, and timestamps.</x:v>
+        <x:v>Expose record depth and locale-scoped review state and history.</x:v>
       </x:c>
       <x:c r="E5" s="30" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="F5" s="30" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="G5" s="30" t="str">
         <x:v>Frontend</x:v>
@@ -918,19 +918,19 @@
         <x:v>S</x:v>
       </x:c>
       <x:c r="K5" s="30" t="str">
-        <x:v>Review metadata</x:v>
+        <x:v>Deployed localization review contract and Record API</x:v>
       </x:c>
       <x:c r="L5" s="30" t="str">
-        <x:v>Add a compact review section for latest agent research, latest human review, created date, and updated date.</x:v>
+        <x:v>Show record depth and the resolved locale's current review state and date to all users. Let authenticated reviewers update review state and note and inspect review history across locales; keep reviewer identity and notes out of public responses.</x:v>
       </x:c>
       <x:c r="M5" s="30" t="str">
-        <x:v>Reviewer can tell whether a record is agent-researched, human-reviewed, stale, or needs revision from User View.</x:v>
+        <x:v>User View shows record depth plus the displayed locale's review state and date. Authorized reviewers can update state and note and inspect reviewer, date, and note history; public users can inspect state, date, and history without private reviewer identity or notes.</x:v>
       </x:c>
       <x:c r="N5" s="30" t="str">
         <x:v>QA Passed</x:v>
       </x:c>
       <x:c r="O5" s="21" t="str">
-        <x:v>Useful for team accountability.</x:v>
+        <x:v>Production smoke verified revision history and review authorization behavior.</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="56" customHeight="1">
@@ -1018,7 +1018,7 @@
         <x:v>Backfill route records, source refs, contract refs, delivery formats, route caveats, and supported tool metadata.</x:v>
       </x:c>
       <x:c r="M7" s="30" t="str">
-        <x:v>Priority systems return complete route metadata through API and MCP, with planned routes separated from live routes.</x:v>
+        <x:v>Priority systems return complete route metadata through the API, with planned routes separated from live routes.</x:v>
       </x:c>
       <x:c r="N7" s="30" t="str">
         <x:v>QA Passed</x:v>
@@ -1082,7 +1082,7 @@
         <x:v>Release 2</x:v>
       </x:c>
       <x:c r="C9" s="30" t="str">
-        <x:v>MCP portal hardening</x:v>
+        <x:v>Portal API hardening</x:v>
       </x:c>
       <x:c r="D9" s="30" t="str">
         <x:v>Make Ryu reliable as a discovery and routing portal.</x:v>
@@ -1106,13 +1106,13 @@
         <x:v>M</x:v>
       </x:c>
       <x:c r="K9" s="30" t="str">
-        <x:v>Existing list/search/get tools</x:v>
+        <x:v>Existing portal API endpoints</x:v>
       </x:c>
       <x:c r="L9" s="30" t="str">
         <x:v>Confirm query parameters, route inclusion behavior, response schema, error handling, and example prompts for system discovery.</x:v>
       </x:c>
       <x:c r="M9" s="30" t="str">
-        <x:v>list_systems, search_systems, and get_system pass smoke tests and return enough route/source/caveat metadata for Deeptime.</x:v>
+        <x:v>The portal API endpoints pass smoke tests and return enough route/source/caveat metadata for Deeptime.</x:v>
       </x:c>
       <x:c r="N9" s="30" t="str">
         <x:v>QA Passed</x:v>
@@ -1368,16 +1368,16 @@
         <x:v>2026-08-24 to 2026-09-13</x:v>
       </x:c>
       <x:c r="E2" s="29" t="str">
-        <x:v>Priority list approved</x:v>
+        <x:v>Priority research queue and record contract approved</x:v>
       </x:c>
       <x:c r="F2" s="29" t="str">
-        <x:v>Rich records and audit-facing UI shipped</x:v>
+        <x:v>Approved rich-record batch applied and read-verified; descriptor evidence and locale review history are available in User View</x:v>
       </x:c>
       <x:c r="G2" s="29" t="str">
-        <x:v>Scope creep in record depth</x:v>
+        <x:v>Scope expansion beyond the approved priority queue</x:v>
       </x:c>
       <x:c r="H2" s="19" t="str">
-        <x:v>Walk through six source-backed systems</x:v>
+        <x:v>Walk through a surviving priority system's descriptors, evidence, record depth, and review history</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="58" customHeight="1">
@@ -1397,7 +1397,7 @@
         <x:v>Tool record archetype accepted</x:v>
       </x:c>
       <x:c r="F3" s="30" t="str">
-        <x:v>Priority route records work through API/MCP</x:v>
+        <x:v>Priority route records work through the API</x:v>
       </x:c>
       <x:c r="G3" s="30" t="str">
         <x:v>Ambiguous route status definitions</x:v>
@@ -1469,7 +1469,7 @@
         <x:v>Release Gate</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" ht="54" customHeight="1">
+    <x:row r="2" ht="84" customHeight="1">
       <x:c r="A2" s="18" t="str">
         <x:v>R1-F01</x:v>
       </x:c>
@@ -1477,19 +1477,19 @@
         <x:v>Record backlog triage</x:v>
       </x:c>
       <x:c r="C2" s="29" t="str">
-        <x:v>Priority list is approved, each selected record has an owner and target review state, and deferred records are explicitly marked.</x:v>
+        <x:v>The approved queue names and orders the priority systems, assigns a primary worker, sets the target depth and review state, keeps supporting identities thin or stub, and records removals or deferrals.</x:v>
       </x:c>
       <x:c r="D2" s="29" t="str">
-        <x:v>Representative user path is verified manually and no critical UI copy is hidden or clipped.</x:v>
+        <x:v>The research queue and current scope identify the main records, supporting identities, primary workers, and removed or deferred items.</x:v>
       </x:c>
       <x:c r="E2" s="29" t="str">
-        <x:v>Depends on Existing Ryu DB</x:v>
+        <x:v>Approved priority research queue and record-shape prerequisite</x:v>
       </x:c>
       <x:c r="F2" s="19" t="str">
         <x:v>Spec Approved</x:v>
       </x:c>
     </x:row>
-    <x:row r="3" ht="54" customHeight="1">
+    <x:row r="3" ht="84" customHeight="1">
       <x:c r="A3" s="20" t="str">
         <x:v>R1-F02</x:v>
       </x:c>
@@ -1497,19 +1497,19 @@
         <x:v>Rich record backfill</x:v>
       </x:c>
       <x:c r="C3" s="30" t="str">
-        <x:v>At least six priority systems have source-backed rich records and no unresolved source refs in visible user-facing fields.</x:v>
+        <x:v>Every approved main record passes live validateOnly with a fresh precondition, applies and reads back exactly, has six complete agent_researched localizations, complete source-reference coverage, qualifying gallery evidence, and fully evidenced incident relationships; supporting identities remain thin or stub.</x:v>
       </x:c>
       <x:c r="D3" s="30" t="str">
-        <x:v>Representative user path is verified manually and no critical UI copy is hidden or clipped.</x:v>
+        <x:v>A reviewer can open a completed system in User View and inspect its localized profile, evidence, gallery, access, metrics, and connections.</x:v>
       </x:c>
       <x:c r="E3" s="30" t="str">
-        <x:v>Depends on R1-F01</x:v>
+        <x:v>Production application report and validation manifest</x:v>
       </x:c>
       <x:c r="F3" s="21" t="str">
         <x:v>QA Passed</x:v>
       </x:c>
     </x:row>
-    <x:row r="4" ht="54" customHeight="1">
+    <x:row r="4" ht="84" customHeight="1">
       <x:c r="A4" s="20" t="str">
         <x:v>R1-F03</x:v>
       </x:c>
@@ -1517,19 +1517,19 @@
         <x:v>Data record visibility</x:v>
       </x:c>
       <x:c r="C4" s="30" t="str">
-        <x:v>Reviewer can verify every visible data type, format, and standard without opening raw fields.</x:v>
+        <x:v>A reviewer can inspect each displayed descriptor's approved label, category, localized description, and resolved source evidence, or the standards gap, without opening Raw Fields.</x:v>
       </x:c>
       <x:c r="D4" s="30" t="str">
-        <x:v>Representative user path is verified manually and no critical UI copy is hidden or clipped.</x:v>
+        <x:v>Keyboard or pointer focus on a descriptor reveals its localized description and source evidence; a missing standard shows the recorded research gap.</x:v>
       </x:c>
       <x:c r="E4" s="30" t="str">
-        <x:v>Depends on Data descriptors already exist</x:v>
+        <x:v>Shared descriptor contract and production smoke evidence</x:v>
       </x:c>
       <x:c r="F4" s="21" t="str">
         <x:v>QA Passed</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" ht="54" customHeight="1">
+    <x:row r="5" ht="84" customHeight="1">
       <x:c r="A5" s="20" t="str">
         <x:v>R1-F04</x:v>
       </x:c>
@@ -1537,13 +1537,13 @@
         <x:v>Review trail surface</x:v>
       </x:c>
       <x:c r="C5" s="30" t="str">
-        <x:v>Reviewer can tell whether a record is agent-researched, human-reviewed, stale, or needs revision from User View.</x:v>
+        <x:v>User View shows record depth plus the displayed locale's review state and date. Authorized reviewers can update state and note and inspect reviewer, date, and note history; public users can inspect state, date, and history without private reviewer identity or notes.</x:v>
       </x:c>
       <x:c r="D5" s="30" t="str">
-        <x:v>Representative user path is verified manually and no critical UI copy is hidden or clipped.</x:v>
+        <x:v>Public view shows review state and date without private identity or notes; authenticated review view exposes controls and the cross-locale revision history.</x:v>
       </x:c>
       <x:c r="E5" s="30" t="str">
-        <x:v>Depends on Review metadata</x:v>
+        <x:v>Localization review contract and production smoke evidence</x:v>
       </x:c>
       <x:c r="F5" s="21" t="str">
         <x:v>QA Passed</x:v>
@@ -1577,7 +1577,7 @@
         <x:v>Tool record backfill</x:v>
       </x:c>
       <x:c r="C7" s="30" t="str">
-        <x:v>Priority systems return complete route metadata through API and MCP, with planned routes separated from live routes.</x:v>
+        <x:v>Priority systems return complete route metadata through the API, with planned routes separated from live routes.</x:v>
       </x:c>
       <x:c r="D7" s="30" t="str">
         <x:v>Representative user path is verified manually and no critical UI copy is hidden or clipped.</x:v>
@@ -1614,16 +1614,16 @@
         <x:v>R2-F04</x:v>
       </x:c>
       <x:c r="B9" s="30" t="str">
-        <x:v>MCP portal hardening</x:v>
+        <x:v>Portal API hardening</x:v>
       </x:c>
       <x:c r="C9" s="30" t="str">
-        <x:v>list_systems, search_systems, and get_system pass smoke tests and return enough route/source/caveat metadata for Deeptime.</x:v>
+        <x:v>The portal API endpoints pass smoke tests and return enough route/source/caveat metadata for Deeptime.</x:v>
       </x:c>
       <x:c r="D9" s="30" t="str">
         <x:v>Representative user path is verified manually and no critical UI copy is hidden or clipped.</x:v>
       </x:c>
       <x:c r="E9" s="30" t="str">
-        <x:v>Depends on Existing list/search/get tools</x:v>
+        <x:v>Depends on Existing portal API endpoints</x:v>
       </x:c>
       <x:c r="F9" s="21" t="str">
         <x:v>QA Passed</x:v>
@@ -1790,10 +1790,10 @@
         <x:v>46262</x:v>
       </x:c>
       <x:c r="F3" s="30" t="str">
-        <x:v>Cap Release 1 to named priority systems and defer the rest.</x:v>
+        <x:v>Scope was capped to the approved priority queue; OceanTeacher's removal was recorded and supporting identities remained thin or stub.</x:v>
       </x:c>
       <x:c r="G3" s="21" t="str">
-        <x:v>Open</x:v>
+        <x:v>Closed</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="52" customHeight="1">

</xml_diff>